<commit_message>
Added basic merge functionalioty and added generic feedback loading from a file
</commit_message>
<xml_diff>
--- a/data/generic-feedbacks.xlsx
+++ b/data/generic-feedbacks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stummuac-my.sharepoint.com/personal/55147483_ad_mmu_ac_uk/Documents/Apps/test data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Physc\Documents\J4S Intern Module Helper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{481B74F1-92A7-4A75-9F0F-B2863A28DB4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{205FC0B6-4BF7-4504-A82C-2092250A802F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FCE2F56-460D-43E0-9CAB-81F517091D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2175" yWindow="4260" windowWidth="21600" windowHeight="11340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,82 +25,73 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>Mark Range</t>
-  </si>
-  <si>
-    <t>General Feedback 2</t>
-  </si>
-  <si>
-    <t>General Feedback 1</t>
-  </si>
-  <si>
-    <t>General Feedback 3</t>
-  </si>
-  <si>
-    <t>0-39</t>
-  </si>
-  <si>
-    <t>40-49</t>
-  </si>
-  <si>
-    <t>50-59</t>
-  </si>
-  <si>
-    <t>60-69</t>
-  </si>
-  <si>
-    <t>70-85</t>
-  </si>
-  <si>
-    <t>85-100</t>
-  </si>
-  <si>
-    <t>You didn't make enough effort to pass this module.</t>
-  </si>
-  <si>
-    <t>You didn't do well in Part 1.</t>
-  </si>
-  <si>
-    <t>You didn't do well in Part 2.</t>
-  </si>
-  <si>
-    <t>Code quality is low, with limited execution and tool utilisation.</t>
-  </si>
-  <si>
-    <t>Code quality is satisfactory, executing essential test cases.</t>
-  </si>
-  <si>
-    <t>Code is efficient, including the majority of test cases and employing basic tools.</t>
-  </si>
-  <si>
-    <t>Code quality is high, with extensive test execution and effective tool utilisation (e.g. Parameterized Tests).</t>
-  </si>
-  <si>
-    <t>Code quality is exceptional/professional, with full test execution and optimal use of advanced tools (e.g. Parameterized Tests utilising external test data).</t>
-  </si>
-  <si>
-    <t>The overall quality is low.</t>
-  </si>
-  <si>
-    <t>The overall quality is satisfactory.</t>
-  </si>
-  <si>
-    <t>The majority is good.</t>
-  </si>
-  <si>
-    <t>Well-presented work.</t>
-  </si>
-  <si>
-    <t>Excellent work.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t>0-30</t>
+  </si>
+  <si>
+    <t>Marks</t>
+  </si>
+  <si>
+    <t>Feedback</t>
+  </si>
+  <si>
+    <t>Your participation and effort in the unit are appreciated. Although your score indicates some challenges, you’ve shown perseverance by coming this far. To improve, concentrate on revisiting Q1 (numeracy) and Q3 . Keep a positive mindset and  continue striving—you have the ability to improve with dedicated effort!</t>
+  </si>
+  <si>
+    <t>30-34</t>
+  </si>
+  <si>
+    <t>35-39</t>
+  </si>
+  <si>
+    <t>Your dedication to the coursework is appreciated, and it's great to see you engaging with the material. To enhance your performance, consider revisiting Q2  and Q6 . Stay positive and keep striving—you have the potential to do well!</t>
+  </si>
+  <si>
+    <t>Thank you for engaging with the coursework and getting this far. Your effort is valued. To improve your results, work on strengthening your skills in Q4 (data analysis) and Q8 . Keep up the hard work and stay motivated—you’re capable of great progress!</t>
+  </si>
+  <si>
+    <t>40-44</t>
+  </si>
+  <si>
+    <t>I appreciate your efforts and commitment to the unit. Although there is room for improvement, you’ve shown determination. To boost your score, focus on understanding Q1  and Q5 . Keep working hard—you can achieve more with continued effort!</t>
+  </si>
+  <si>
+    <t>45-49</t>
+  </si>
+  <si>
+    <t>65-69</t>
+  </si>
+  <si>
+    <t>Good job on your assignment! You’re on the right track with your understanding. To boost your score, focus on improving your responses in Q2 (numeracy) and Q4 (data analysis). Keep up the hard work and aim higher!</t>
+  </si>
+  <si>
+    <t>75-79</t>
+  </si>
+  <si>
+    <t>80-84</t>
+  </si>
+  <si>
+    <t>Great effort! You’ve demonstrated a solid understanding of the coursework. To reach the next level, review Q3 (numeracy) and Q4 (data analysis) where you lost some marks. Keep up the excellent work!</t>
+  </si>
+  <si>
+    <t>Well done on your assignment! Your performance shows a good comprehension of the topics. However, you can enhance your score by revisiting Q4 (data interpretation) and Q7 (numeracy). Stay motivated and continue improving!</t>
+  </si>
+  <si>
+    <t>Thank you for your effort and engagement with the unit. You’ve made it this far, which is commendable. To improve, focus on strengthening your understanding of Q3  and Q7 (data analysis). Keep pushing forward—you’re on the right path!</t>
+  </si>
+  <si>
+    <t>85-90</t>
+  </si>
+  <si>
+    <t>Fantastic job on your assignment! Your hard work is evident, and you have a strong grasp of the material. To further improve, focus on refining your answers in Q2 (data analysis) and Q5 (Numeracy). Keep pushing forward!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,6 +104,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0D0D0D"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -135,10 +138,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -420,102 +430,107 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="255.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" customWidth="1"/>
     <col min="4" max="4" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
updated some extra files mainly the xlsx ones
</commit_message>
<xml_diff>
--- a/data/generic-feedbacks.xlsx
+++ b/data/generic-feedbacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Physc\Documents\J4S Intern Module Helper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FCE2F56-460D-43E0-9CAB-81F517091D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5834533-F5CA-437B-94FB-E7FCFD617E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20235" yWindow="8925" windowWidth="29010" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>